<commit_message>
housekeep-db: excel files bugs fixed
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v1.3.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v1.3.0-en_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tools/ecuacion-tool-housekeep-db/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F78598C-5185-9946-ADEE-346FDE6D42B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{064403C5-DD23-3F4C-8144-60127F371CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16640" activeTab="5" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
   </bookViews>
   <sheets>
     <sheet name="change log" sheetId="8" r:id="rId1"/>
@@ -18,8 +18,8 @@
     <sheet name="dropdown" sheetId="15" state="hidden" r:id="rId3"/>
     <sheet name="DB Connection Settings" sheetId="4" r:id="rId4"/>
     <sheet name="Housekeep DB Settings" sheetId="10" r:id="rId5"/>
-    <sheet name="Related Table Settings" sheetId="14" r:id="rId6"/>
-    <sheet name="Search Condition Settings" sheetId="12" r:id="rId7"/>
+    <sheet name="Search Condition Settings" sheetId="12" r:id="rId6"/>
+    <sheet name="Related Table Settings" sheetId="14" r:id="rId7"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId8"/>
@@ -48,8 +48,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="73">
   <si>
     <t>value</t>
     <phoneticPr fontId="1"/>
@@ -269,6 +291,9 @@
   </si>
   <si>
     <t>housekeep-db: v15</t>
+  </si>
+  <si>
+    <t>VLOOKUP([@処理ID],テーブル32[[処理ID]:[論理廃止 / 削除（内部値）]],4,FALSE)</t>
   </si>
 </sst>
 </file>
@@ -503,26 +528,26 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -541,6 +566,76 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
         <scheme val="minor"/>
       </font>
     </dxf>
@@ -739,6 +834,291 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -975,361 +1355,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
@@ -1484,107 +1509,107 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D5" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D5" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A3:D5" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="Date" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="Version" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="Notes" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="Updated By" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="Date" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="Version" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="Notes" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="Updated By" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="A1:B3" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="A5:I6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB Connection ID" dataDxfId="40" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="Driver Name" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="Connection URL: Protocol" dataDxfId="38" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="Connection URL: Server" dataDxfId="37" dataCellStyle="標準 2"/>
-    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="Connection URL: Port" dataDxfId="36" dataCellStyle="標準 2"/>
-    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="Connection URL: Database" dataDxfId="35" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="Connection URL: Schema" dataDxfId="34" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="Username" dataDxfId="33" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="Password" dataDxfId="32" dataCellStyle="標準 2"/>
+    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB Connection ID" dataDxfId="28" dataCellStyle="標準 2"/>
+    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="Driver Name" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="Connection URL: Protocol" dataDxfId="26" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="Connection URL: Server" dataDxfId="25" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="Connection URL: Port" dataDxfId="24" dataCellStyle="標準 2"/>
+    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="Connection URL: Database" dataDxfId="23" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="Connection URL: Schema" dataDxfId="22" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="Username" dataDxfId="21" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="Password" dataDxfId="20" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A5:O6" insertRow="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A5:O6" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A5:O6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="29"/>
-    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="28" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Soft / Hard Delete" dataDxfId="27"/>
-    <tableColumn id="15" xr3:uid="{C9A2944C-947B-B844-AE98-12A7D9A1D364}" name="Soft / Hard Delete (internal value)" dataDxfId="26">
-      <calculatedColumnFormula>IF(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE","HARD_DELETE")</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="55"/>
+    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="54" dataCellStyle="標準 2"/>
+    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Soft / Hard Delete" dataDxfId="53"/>
+    <tableColumn id="15" xr3:uid="{C9A2944C-947B-B844-AE98-12A7D9A1D364}" name="Soft / Hard Delete (internal value)" dataDxfId="52">
+      <calculatedColumnFormula array="1">_xlfn.IFS(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Soft / Hard Delete]]="Hard Delete","HARD_DELETE",TRUE,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="25" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="24" dataCellStyle="標準 2"/>
-    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Timestamp Column Name" dataDxfId="22" dataCellStyle="標準 2"/>
-    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="20" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="19" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="18" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="Soft Delete: Update User ID Column Name" dataDxfId="17" dataCellStyle="標準 2"/>
-    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="16" dataCellStyle="標準 2"/>
-    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="Soft Delete: Update User ID Column Value" dataDxfId="15" dataCellStyle="標準 2"/>
+    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="51" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="50" dataCellStyle="標準 2"/>
+    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Timestamp Column Name" dataDxfId="48" dataCellStyle="標準 2"/>
+    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="46" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="45" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="44" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="Soft Delete: Update User ID Column Name" dataDxfId="43" dataCellStyle="標準 2"/>
+    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="42" dataCellStyle="標準 2"/>
+    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="Soft Delete: Update User ID Column Value" dataDxfId="41" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A5:M6" insertRow="1" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
-  <autoFilter ref="A5:M6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{65C86A53-0A13-8F47-916D-E06475BCECE3}" name="Task ID" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{5FFE67A8-33A0-B648-BE60-A87A07B8D65D}" name="Soft / Hard Delete (internal value)" dataDxfId="11">
-      <calculatedColumnFormula>VLOOKUP(テーブル3236[[#This Row],[Task ID]],テーブル32[[Task ID]:[Soft / Hard Delete (internal value)]],4,FALSE)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{987F2B9C-94EA-9F41-A4C1-6D7606B12BAC}" name="Related Table Process Pattern" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{B871A9E9-220D-F74C-A1C5-BED1ED6DD954}" name="Related Table Process Pattern (internal value)" dataDxfId="9">
-      <calculatedColumnFormula array="1">_xlfn.IFS(テーブル3236[[#This Row],[Related Table Process Pattern]]="Delete","DELETE",テーブル3236[[#This Row],[Related Table Process Pattern]]="Check and Skip Delete","CHECK_AND_SKIP_DELETE",TRUE,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{5E73C8D1-B2FA-854B-BEBB-60B6E93A2638}" name="Target Table Column Name" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{3B40126A-13DD-E04B-A86B-9387EB6006A1}" name="Related Table Name" dataDxfId="7" dataCellStyle="標準 2"/>
-    <tableColumn id="3" xr3:uid="{59ED585B-1BCF-DB41-A333-2655E74C710D}" name="Related Table ID Column Name" dataDxfId="6" dataCellStyle="標準 2"/>
-    <tableColumn id="14" xr3:uid="{75144EA6-AFC2-3646-9A0E-DD4A2D917411}" name="Related Table ID Column Literal Symbol" dataDxfId="5" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{684AF203-54CE-5A42-8441-2636BF604DAF}" name="Soft Delete Column Name" dataDxfId="4" dataCellStyle="標準 2"/>
-    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="3" dataCellStyle="標準 2"/>
-    <tableColumn id="6" xr3:uid="{59287FEB-061F-B946-B814-312CDD2F482D}" name="Soft Delete: Update User ID Column Name" dataDxfId="2" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{E0734288-8DC3-C342-98A6-DBC50A55CEF9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="1" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{D5E8A958-B06D-554D-B183-49DD307AC86A}" name="Soft Delete: Update User ID Column Value" dataDxfId="0" dataCellStyle="標準 2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A5:D6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="Task ID" dataDxfId="3" dataCellStyle="標準 2"/>
+    <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="Search Condition Column Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{511F37DB-74E3-394C-9204-B1C6CA623CD0}" name="Search Condtion Column Literal Symbol" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{2F474AF9-6428-D446-9D8C-0FEF2C86FE1D}" name="Search Condition Column Value" dataDxfId="0" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="57">
-  <autoFilter ref="A5:D6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="Task ID" dataDxfId="56" dataCellStyle="標準 2"/>
-    <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="Search Condition Column Name" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{511F37DB-74E3-394C-9204-B1C6CA623CD0}" name="Search Condtion Column Literal Symbol" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{2F474AF9-6428-D446-9D8C-0FEF2C86FE1D}" name="Search Condition Column Value" dataDxfId="53" dataCellStyle="標準 2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A5:M6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A5:M6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{65C86A53-0A13-8F47-916D-E06475BCECE3}" name="Task ID" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{5FFE67A8-33A0-B648-BE60-A87A07B8D65D}" name="Soft / Hard Delete (internal value)" dataDxfId="16">
+      <calculatedColumnFormula>VLOOKUP(テーブル3236[[#This Row],[Task ID]],テーブル32[[#This Row],[Task ID]:[Soft / Hard Delete (internal value)]],4,FALSE)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{987F2B9C-94EA-9F41-A4C1-6D7606B12BAC}" name="Related Table Process Pattern" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{B871A9E9-220D-F74C-A1C5-BED1ED6DD954}" name="Related Table Process Pattern (internal value)" dataDxfId="14">
+      <calculatedColumnFormula array="1">_xlfn.IFS(テーブル3236[[#This Row],[Related Table Process Pattern]]="Delete","DELETE",テーブル3236[[#This Row],[Related Table Process Pattern]]="Check and Skip Delete","CHECK_AND_SKIP_DELETE",TRUE,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{5E73C8D1-B2FA-854B-BEBB-60B6E93A2638}" name="Target Table Column Name" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{3B40126A-13DD-E04B-A86B-9387EB6006A1}" name="Related Table Name" dataDxfId="12" dataCellStyle="標準 2"/>
+    <tableColumn id="3" xr3:uid="{59ED585B-1BCF-DB41-A333-2655E74C710D}" name="Related Table ID Column Name" dataDxfId="11" dataCellStyle="標準 2"/>
+    <tableColumn id="14" xr3:uid="{75144EA6-AFC2-3646-9A0E-DD4A2D917411}" name="Related Table ID Column Literal Symbol" dataDxfId="10" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{684AF203-54CE-5A42-8441-2636BF604DAF}" name="Soft Delete Column Name" dataDxfId="9" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="8" dataCellStyle="標準 2"/>
+    <tableColumn id="6" xr3:uid="{59287FEB-061F-B946-B814-312CDD2F482D}" name="Soft Delete: Update User ID Column Name" dataDxfId="7" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{E0734288-8DC3-C342-98A6-DBC50A55CEF9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="6" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{D5E8A958-B06D-554D-B183-49DD307AC86A}" name="Soft Delete: Update User ID Column Value" dataDxfId="5" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1931,13 +1956,13 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="29">
+      <c r="A5" s="25">
         <v>46256</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="23" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="11" t="s">
@@ -2152,21 +2177,21 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="24"/>
+      <c r="I4" s="29"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -2272,33 +2297,33 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
       <c r="D4" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="25" t="s">
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
       <c r="K4" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="26" t="s">
+      <c r="L4" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -2350,7 +2375,10 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
       <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="D6" s="8" t="str" cm="1">
+        <f t="array" ref="D6">_xlfn.IFS(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Soft / Hard Delete]]="Hard Delete","HARD_DELETE",TRUE,"")</f>
+        <v/>
+      </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
@@ -2444,8 +2472,81 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E1BEA4-8682-2D4B-83F3-E3D5D9773981}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="37.83203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="7.5" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:D4"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C7" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
+      <formula1>"quotes('),(none)"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A480BCC2-429D-064C-9186-E29D7E93B50F}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
@@ -2491,19 +2592,19 @@
       <c r="D4" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="25" t="s">
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="25"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -2548,9 +2649,15 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
+      <c r="B6" s="8" t="e">
+        <f>VLOOKUP(テーブル3236[[#This Row],[Task ID]],テーブル32[[#This Row],[Task ID]:[Soft / Hard Delete (internal value)]],4,FALSE)</f>
+        <v>#N/A</v>
+      </c>
       <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="D6" s="8" t="str" cm="1">
+        <f t="array" ref="D6">_xlfn.IFS(テーブル3236[[#This Row],[Related Table Process Pattern]]="Delete","DELETE",テーブル3236[[#This Row],[Related Table Process Pattern]]="Check and Skip Delete","CHECK_AND_SKIP_DELETE",TRUE,"")</f>
+        <v/>
+      </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="7"/>
@@ -2597,6 +2704,11 @@
         <v>61</v>
       </c>
       <c r="B11" s="15"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B13" s="6" t="s">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2618,77 +2730,4 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E1BEA4-8682-2D4B-83F3-E3D5D9773981}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="37.83203125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="7.5" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A4:D4"/>
-  </mergeCells>
-  <phoneticPr fontId="1"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C7" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
-      <formula1>"quotes('),(none)"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>